<commit_message>
Arregla acceso y firmas dinámicas en PDFs de calificación e informe de jefatura
</commit_message>
<xml_diff>
--- a/src/fixtures/nomina_prueba_sapd.xlsx
+++ b/src/fixtures/nomina_prueba_sapd.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="95">
   <si>
     <t>N° Personal</t>
   </si>
@@ -137,180 +137,90 @@
     <t>carlos.fuentes@ucm.cl</t>
   </si>
   <si>
-    <t>003</t>
-  </si>
-  <si>
-    <t>20.333.444-5</t>
-  </si>
-  <si>
-    <t>Pedro Andrés Alarcón Rojas</t>
+    <t>005</t>
+  </si>
+  <si>
+    <t>20.555.666-7</t>
+  </si>
+  <si>
+    <t>Roberto Ignacio Jiménez Díaz</t>
   </si>
   <si>
     <t>Depto. Computación e Informática</t>
   </si>
   <si>
+    <t>Profesor Auxiliar</t>
+  </si>
+  <si>
+    <t>01/08/2020</t>
+  </si>
+  <si>
+    <t>auxiliar</t>
+  </si>
+  <si>
+    <t>roberto.jimenez@ucm.cl</t>
+  </si>
+  <si>
+    <t>009</t>
+  </si>
+  <si>
+    <t>20.999.000-1</t>
+  </si>
+  <si>
+    <t>Gabriel Antonio Morales Cid</t>
+  </si>
+  <si>
     <t>Profesor</t>
   </si>
   <si>
+    <t>01/03/2018</t>
+  </si>
+  <si>
+    <t>01/03/2020</t>
+  </si>
+  <si>
+    <t>Bueno</t>
+  </si>
+  <si>
+    <t>gabriel.morales@ucm.cl</t>
+  </si>
+  <si>
+    <t>010</t>
+  </si>
+  <si>
+    <t>21.000.111-2</t>
+  </si>
+  <si>
+    <t>Claudia Fernanda Vega Soto</t>
+  </si>
+  <si>
+    <t>Depto. Matemáticas</t>
+  </si>
+  <si>
+    <t>Profesora Titular</t>
+  </si>
+  <si>
+    <t>01/03/2010</t>
+  </si>
+  <si>
     <t>01/03/2014</t>
   </si>
   <si>
-    <t>01/03/2018</t>
-  </si>
-  <si>
-    <t>pedro.alarcon@ucm.cl</t>
-  </si>
-  <si>
-    <t>004</t>
-  </si>
-  <si>
-    <t>20.444.555-6</t>
-  </si>
-  <si>
-    <t>Sandra Beatriz Muñoz Lagos</t>
-  </si>
-  <si>
-    <t>Depto. Matemáticas</t>
-  </si>
-  <si>
-    <t>Profesora</t>
-  </si>
-  <si>
-    <t>01/03/2016</t>
-  </si>
-  <si>
-    <t>01/03/2020</t>
-  </si>
-  <si>
-    <t>sandra.munoz@ucm.cl</t>
-  </si>
-  <si>
-    <t>005</t>
-  </si>
-  <si>
-    <t>20.555.666-7</t>
-  </si>
-  <si>
-    <t>Roberto Ignacio Jiménez Díaz</t>
-  </si>
-  <si>
-    <t>Profesor Auxiliar</t>
-  </si>
-  <si>
-    <t>01/08/2020</t>
-  </si>
-  <si>
-    <t>auxiliar</t>
-  </si>
-  <si>
-    <t>roberto.jimenez@ucm.cl</t>
-  </si>
-  <si>
-    <t>006</t>
-  </si>
-  <si>
-    <t>20.666.777-8</t>
-  </si>
-  <si>
-    <t>Ana Patricia Martínez Pérez</t>
-  </si>
-  <si>
-    <t>01/03/2012</t>
-  </si>
-  <si>
-    <t>Bueno</t>
-  </si>
-  <si>
-    <t>ana.martinez@ucm.cl</t>
-  </si>
-  <si>
-    <t>007</t>
-  </si>
-  <si>
-    <t>20.777.888-9</t>
-  </si>
-  <si>
-    <t>Luis Hernán Contreras Bravo</t>
+    <t>claudia.vega@ucm.cl</t>
+  </si>
+  <si>
+    <t>011</t>
+  </si>
+  <si>
+    <t>21.111.222-3</t>
+  </si>
+  <si>
+    <t>Diego Mauricio Espinoza Araya</t>
   </si>
   <si>
     <t>Contrata</t>
   </si>
   <si>
-    <t>Profesor Instructor</t>
-  </si>
-  <si>
-    <t>Académico Hora</t>
-  </si>
-  <si>
-    <t>01/03/2025</t>
-  </si>
-  <si>
-    <t>instructor</t>
-  </si>
-  <si>
-    <t>luis.contreras@ucm.cl</t>
-  </si>
-  <si>
-    <t>008</t>
-  </si>
-  <si>
-    <t>20.888.999-0</t>
-  </si>
-  <si>
-    <t>Valentina Paz Torres Ríos</t>
-  </si>
-  <si>
-    <t>Profesora Auxiliar</t>
-  </si>
-  <si>
-    <t>01/08/2021</t>
-  </si>
-  <si>
-    <t>valentina.torres@ucm.cl</t>
-  </si>
-  <si>
-    <t>009</t>
-  </si>
-  <si>
-    <t>20.999.000-1</t>
-  </si>
-  <si>
-    <t>Gabriel Antonio Morales Cid</t>
-  </si>
-  <si>
-    <t>01/08/2025</t>
-  </si>
-  <si>
-    <t>gabriel.morales@ucm.cl</t>
-  </si>
-  <si>
-    <t>010</t>
-  </si>
-  <si>
-    <t>21.000.111-2</t>
-  </si>
-  <si>
-    <t>Claudia Fernanda Vega Soto</t>
-  </si>
-  <si>
-    <t>Profesora Titular</t>
-  </si>
-  <si>
-    <t>01/03/2010</t>
-  </si>
-  <si>
-    <t>claudia.vega@ucm.cl</t>
-  </si>
-  <si>
-    <t>011</t>
-  </si>
-  <si>
-    <t>21.111.222-3</t>
-  </si>
-  <si>
-    <t>Diego Mauricio Espinoza Araya</t>
-  </si>
-  <si>
     <t>01/08/2019</t>
   </si>
   <si>
@@ -320,21 +230,6 @@
     <t>diego.espinoza@ucm.cl</t>
   </si>
   <si>
-    <t>012</t>
-  </si>
-  <si>
-    <t>21.222.333-4</t>
-  </si>
-  <si>
-    <t>Francisca Isabel Núñez Bravo</t>
-  </si>
-  <si>
-    <t>01/03/2022</t>
-  </si>
-  <si>
-    <t>francisca.nunez@ucm.cl</t>
-  </si>
-  <si>
     <t>22.111.222-3</t>
   </si>
   <si>
@@ -389,43 +284,22 @@
     <t>patricia.lagos@ucm.cl</t>
   </si>
   <si>
-    <t>22.444.555-6</t>
-  </si>
-  <si>
-    <t>Fernando Andrés Muñoz Pérez</t>
+    <t>22.555.666-7</t>
+  </si>
+  <si>
+    <t>Paula Andrea Morales Vega</t>
+  </si>
+  <si>
+    <t>Depto. Silvicultura</t>
+  </si>
+  <si>
+    <t>01/03/2011</t>
   </si>
   <si>
     <t>01/03/2015</t>
   </si>
   <si>
-    <t>01/03/2019</t>
-  </si>
-  <si>
-    <t>fernando.munoz@ucm.cl</t>
-  </si>
-  <si>
-    <t>22.555.666-7</t>
-  </si>
-  <si>
-    <t>Paula Andrea Morales Vega</t>
-  </si>
-  <si>
-    <t>Depto. Silvicultura</t>
-  </si>
-  <si>
-    <t>01/03/2011</t>
-  </si>
-  <si>
     <t>paula.morales@ucm.cl</t>
-  </si>
-  <si>
-    <t>22.666.777-8</t>
-  </si>
-  <si>
-    <t>Camilo Esteban Ríos Bravo</t>
-  </si>
-  <si>
-    <t>camilo.rios@ucm.cl</t>
   </si>
 </sst>
 </file>
@@ -775,7 +649,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="true" style="0"/>
@@ -970,10 +844,10 @@
         <v>24</v>
       </c>
       <c r="K4" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="L4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="Q4" t="s">
         <v>47</v>
@@ -996,16 +870,16 @@
         <v>21</v>
       </c>
       <c r="F5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G5" t="s">
         <v>51</v>
-      </c>
-      <c r="G5" t="s">
-        <v>52</v>
       </c>
       <c r="H5" t="s">
         <v>35</v>
       </c>
       <c r="I5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J5">
         <v>24</v>
@@ -1014,6 +888,12 @@
         <v>37</v>
       </c>
       <c r="L5" t="s">
+        <v>53</v>
+      </c>
+      <c r="M5">
+        <v>3.6</v>
+      </c>
+      <c r="N5" t="s">
         <v>54</v>
       </c>
       <c r="Q5" t="s">
@@ -1037,63 +917,63 @@
         <v>21</v>
       </c>
       <c r="F6" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="G6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H6" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="I6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J6">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="K6" t="s">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="L6" t="s">
-        <v>60</v>
-      </c>
-      <c r="O6">
-        <v>4.6</v>
-      </c>
-      <c r="P6" t="s">
+        <v>62</v>
+      </c>
+      <c r="M6">
+        <v>4.8</v>
+      </c>
+      <c r="N6" t="s">
         <v>28</v>
       </c>
       <c r="Q6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D7" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="E7" t="s">
         <v>21</v>
       </c>
       <c r="F7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" t="s">
         <v>51</v>
-      </c>
-      <c r="G7" t="s">
-        <v>52</v>
       </c>
       <c r="H7" t="s">
         <v>35</v>
       </c>
       <c r="I7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="J7">
         <v>24</v>
@@ -1102,192 +982,192 @@
         <v>37</v>
       </c>
       <c r="L7" t="s">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="M7">
-        <v>4.0</v>
+        <v>3.2</v>
       </c>
       <c r="N7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:17">
-      <c r="A8" t="s">
-        <v>69</v>
+      <c r="A8">
+        <v>101</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D8" t="s">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="E8" t="s">
-        <v>21</v>
+        <v>73</v>
       </c>
       <c r="F8" t="s">
-        <v>43</v>
+        <v>74</v>
       </c>
       <c r="G8" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="H8" t="s">
-        <v>74</v>
+        <v>35</v>
       </c>
       <c r="I8" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="J8">
         <v>24</v>
       </c>
       <c r="K8" t="s">
+        <v>37</v>
+      </c>
+      <c r="L8" t="s">
+        <v>52</v>
+      </c>
+      <c r="M8">
+        <v>4.1</v>
+      </c>
+      <c r="N8" t="s">
+        <v>75</v>
+      </c>
+      <c r="O8">
+        <v>4.0</v>
+      </c>
+      <c r="P8" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q8" t="s">
         <v>76</v>
-      </c>
-      <c r="L8" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:17">
-      <c r="A9" t="s">
+      <c r="A9">
+        <v>102</v>
+      </c>
+      <c r="B9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" t="s">
         <v>78</v>
-      </c>
-      <c r="B9" t="s">
-        <v>79</v>
-      </c>
-      <c r="C9" t="s">
-        <v>80</v>
       </c>
       <c r="D9" t="s">
         <v>20</v>
       </c>
       <c r="E9" t="s">
-        <v>21</v>
+        <v>73</v>
       </c>
       <c r="F9" t="s">
+        <v>79</v>
+      </c>
+      <c r="G9" t="s">
         <v>51</v>
       </c>
-      <c r="G9" t="s">
-        <v>81</v>
-      </c>
       <c r="H9" t="s">
-        <v>74</v>
+        <v>35</v>
       </c>
       <c r="I9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="J9">
         <v>24</v>
       </c>
       <c r="K9" t="s">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="L9" t="s">
+        <v>81</v>
+      </c>
+      <c r="M9">
+        <v>4.4</v>
+      </c>
+      <c r="N9" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q9" t="s">
         <v>82</v>
-      </c>
-      <c r="M9">
-        <v>3.8</v>
-      </c>
-      <c r="N9" t="s">
-        <v>67</v>
-      </c>
-      <c r="O9">
-        <v>4.0</v>
-      </c>
-      <c r="P9" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="10" spans="1:17">
-      <c r="A10" t="s">
+      <c r="A10">
+        <v>103</v>
+      </c>
+      <c r="B10" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" t="s">
         <v>84</v>
-      </c>
-      <c r="B10" t="s">
-        <v>85</v>
-      </c>
-      <c r="C10" t="s">
-        <v>86</v>
       </c>
       <c r="D10" t="s">
         <v>20</v>
       </c>
       <c r="E10" t="s">
-        <v>21</v>
+        <v>73</v>
       </c>
       <c r="F10" t="s">
-        <v>43</v>
+        <v>85</v>
       </c>
       <c r="G10" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="H10" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="I10" t="s">
-        <v>46</v>
+        <v>86</v>
       </c>
       <c r="J10">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="K10" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="L10" t="s">
         <v>87</v>
       </c>
       <c r="M10">
-        <v>3.6</v>
+        <v>4.6</v>
       </c>
       <c r="N10" t="s">
-        <v>67</v>
-      </c>
-      <c r="O10">
-        <v>3.9</v>
-      </c>
-      <c r="P10" t="s">
-        <v>67</v>
+        <v>28</v>
       </c>
       <c r="Q10" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="11" spans="1:17">
-      <c r="A11" t="s">
+      <c r="A11">
+        <v>105</v>
+      </c>
+      <c r="B11" t="s">
         <v>89</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>90</v>
-      </c>
-      <c r="C11" t="s">
-        <v>91</v>
       </c>
       <c r="D11" t="s">
         <v>20</v>
       </c>
       <c r="E11" t="s">
-        <v>21</v>
+        <v>73</v>
       </c>
       <c r="F11" t="s">
-        <v>51</v>
+        <v>91</v>
       </c>
       <c r="G11" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="H11" t="s">
         <v>24</v>
       </c>
       <c r="I11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J11">
         <v>40</v>
@@ -1296,404 +1176,22 @@
         <v>26</v>
       </c>
       <c r="L11" t="s">
-        <v>45</v>
+        <v>93</v>
       </c>
       <c r="M11">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="N11" t="s">
         <v>28</v>
       </c>
+      <c r="O11">
+        <v>4.6</v>
+      </c>
+      <c r="P11" t="s">
+        <v>28</v>
+      </c>
       <c r="Q11" t="s">
         <v>94</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17">
-      <c r="A12" t="s">
-        <v>95</v>
-      </c>
-      <c r="B12" t="s">
-        <v>96</v>
-      </c>
-      <c r="C12" t="s">
-        <v>97</v>
-      </c>
-      <c r="D12" t="s">
-        <v>72</v>
-      </c>
-      <c r="E12" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" t="s">
-        <v>43</v>
-      </c>
-      <c r="G12" t="s">
-        <v>44</v>
-      </c>
-      <c r="H12" t="s">
-        <v>35</v>
-      </c>
-      <c r="I12" t="s">
-        <v>98</v>
-      </c>
-      <c r="J12">
-        <v>24</v>
-      </c>
-      <c r="K12" t="s">
-        <v>37</v>
-      </c>
-      <c r="L12" t="s">
-        <v>98</v>
-      </c>
-      <c r="M12">
-        <v>3.2</v>
-      </c>
-      <c r="N12" t="s">
-        <v>99</v>
-      </c>
-      <c r="O12">
-        <v>3.5</v>
-      </c>
-      <c r="P12" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17">
-      <c r="A13" t="s">
-        <v>101</v>
-      </c>
-      <c r="B13" t="s">
-        <v>102</v>
-      </c>
-      <c r="C13" t="s">
-        <v>103</v>
-      </c>
-      <c r="D13" t="s">
-        <v>20</v>
-      </c>
-      <c r="E13" t="s">
-        <v>21</v>
-      </c>
-      <c r="F13" t="s">
-        <v>51</v>
-      </c>
-      <c r="G13" t="s">
-        <v>81</v>
-      </c>
-      <c r="H13" t="s">
-        <v>35</v>
-      </c>
-      <c r="I13" t="s">
-        <v>104</v>
-      </c>
-      <c r="J13">
-        <v>24</v>
-      </c>
-      <c r="K13" t="s">
-        <v>61</v>
-      </c>
-      <c r="L13" t="s">
-        <v>104</v>
-      </c>
-      <c r="O13">
-        <v>3.7</v>
-      </c>
-      <c r="P13" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q13" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17">
-      <c r="A14">
-        <v>101</v>
-      </c>
-      <c r="B14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" t="s">
-        <v>107</v>
-      </c>
-      <c r="D14" t="s">
-        <v>20</v>
-      </c>
-      <c r="E14" t="s">
-        <v>108</v>
-      </c>
-      <c r="F14" t="s">
-        <v>109</v>
-      </c>
-      <c r="G14" t="s">
-        <v>34</v>
-      </c>
-      <c r="H14" t="s">
-        <v>35</v>
-      </c>
-      <c r="I14" t="s">
-        <v>45</v>
-      </c>
-      <c r="J14">
-        <v>24</v>
-      </c>
-      <c r="K14" t="s">
-        <v>37</v>
-      </c>
-      <c r="L14" t="s">
-        <v>46</v>
-      </c>
-      <c r="M14">
-        <v>4.1</v>
-      </c>
-      <c r="N14" t="s">
-        <v>110</v>
-      </c>
-      <c r="O14">
-        <v>4.0</v>
-      </c>
-      <c r="P14" t="s">
-        <v>110</v>
-      </c>
-      <c r="Q14" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17">
-      <c r="A15">
-        <v>102</v>
-      </c>
-      <c r="B15" t="s">
-        <v>112</v>
-      </c>
-      <c r="C15" t="s">
-        <v>113</v>
-      </c>
-      <c r="D15" t="s">
-        <v>20</v>
-      </c>
-      <c r="E15" t="s">
-        <v>108</v>
-      </c>
-      <c r="F15" t="s">
-        <v>114</v>
-      </c>
-      <c r="G15" t="s">
-        <v>44</v>
-      </c>
-      <c r="H15" t="s">
-        <v>35</v>
-      </c>
-      <c r="I15" t="s">
-        <v>115</v>
-      </c>
-      <c r="J15">
-        <v>24</v>
-      </c>
-      <c r="K15" t="s">
-        <v>37</v>
-      </c>
-      <c r="L15" t="s">
-        <v>116</v>
-      </c>
-      <c r="M15">
-        <v>4.4</v>
-      </c>
-      <c r="N15" t="s">
-        <v>110</v>
-      </c>
-      <c r="Q15" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17">
-      <c r="A16">
-        <v>103</v>
-      </c>
-      <c r="B16" t="s">
-        <v>118</v>
-      </c>
-      <c r="C16" t="s">
-        <v>119</v>
-      </c>
-      <c r="D16" t="s">
-        <v>20</v>
-      </c>
-      <c r="E16" t="s">
-        <v>108</v>
-      </c>
-      <c r="F16" t="s">
-        <v>120</v>
-      </c>
-      <c r="G16" t="s">
-        <v>23</v>
-      </c>
-      <c r="H16" t="s">
-        <v>24</v>
-      </c>
-      <c r="I16" t="s">
-        <v>121</v>
-      </c>
-      <c r="J16">
-        <v>40</v>
-      </c>
-      <c r="K16" t="s">
-        <v>26</v>
-      </c>
-      <c r="L16" t="s">
-        <v>122</v>
-      </c>
-      <c r="M16">
-        <v>4.6</v>
-      </c>
-      <c r="N16" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q16" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17">
-      <c r="A17">
-        <v>104</v>
-      </c>
-      <c r="B17" t="s">
-        <v>124</v>
-      </c>
-      <c r="C17" t="s">
-        <v>125</v>
-      </c>
-      <c r="D17" t="s">
-        <v>20</v>
-      </c>
-      <c r="E17" t="s">
-        <v>108</v>
-      </c>
-      <c r="F17" t="s">
-        <v>114</v>
-      </c>
-      <c r="G17" t="s">
-        <v>44</v>
-      </c>
-      <c r="H17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I17" t="s">
-        <v>126</v>
-      </c>
-      <c r="J17">
-        <v>24</v>
-      </c>
-      <c r="K17" t="s">
-        <v>37</v>
-      </c>
-      <c r="L17" t="s">
-        <v>127</v>
-      </c>
-      <c r="M17">
-        <v>3.9</v>
-      </c>
-      <c r="N17" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17">
-      <c r="A18">
-        <v>105</v>
-      </c>
-      <c r="B18" t="s">
-        <v>129</v>
-      </c>
-      <c r="C18" t="s">
-        <v>130</v>
-      </c>
-      <c r="D18" t="s">
-        <v>20</v>
-      </c>
-      <c r="E18" t="s">
-        <v>108</v>
-      </c>
-      <c r="F18" t="s">
-        <v>131</v>
-      </c>
-      <c r="G18" t="s">
-        <v>92</v>
-      </c>
-      <c r="H18" t="s">
-        <v>24</v>
-      </c>
-      <c r="I18" t="s">
-        <v>132</v>
-      </c>
-      <c r="J18">
-        <v>40</v>
-      </c>
-      <c r="K18" t="s">
-        <v>26</v>
-      </c>
-      <c r="L18" t="s">
-        <v>126</v>
-      </c>
-      <c r="M18">
-        <v>4.5</v>
-      </c>
-      <c r="N18" t="s">
-        <v>28</v>
-      </c>
-      <c r="O18">
-        <v>4.6</v>
-      </c>
-      <c r="P18" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q18" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17">
-      <c r="A19">
-        <v>106</v>
-      </c>
-      <c r="B19" t="s">
-        <v>134</v>
-      </c>
-      <c r="C19" t="s">
-        <v>135</v>
-      </c>
-      <c r="D19" t="s">
-        <v>72</v>
-      </c>
-      <c r="E19" t="s">
-        <v>108</v>
-      </c>
-      <c r="F19" t="s">
-        <v>114</v>
-      </c>
-      <c r="G19" t="s">
-        <v>73</v>
-      </c>
-      <c r="H19" t="s">
-        <v>74</v>
-      </c>
-      <c r="I19" t="s">
-        <v>75</v>
-      </c>
-      <c r="J19">
-        <v>24</v>
-      </c>
-      <c r="K19" t="s">
-        <v>76</v>
-      </c>
-      <c r="L19" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q19" t="s">
-        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>